<commit_message>
feat: update 3.2.4 mn
</commit_message>
<xml_diff>
--- a/3.1.4答案/智能健康监测系统数据集.xlsx
+++ b/3.1.4答案/智能健康监测系统数据集.xlsx
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="216" uniqueCount="152">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="216" uniqueCount="153">
   <si>
     <t>时间戳</t>
   </si>
@@ -495,6 +495,10 @@
   </si>
   <si>
     <t>响应时间</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>HOUR</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
 </sst>
@@ -594,7 +598,7 @@
 <file path=xl/pivotCache/pivotCacheDefinition1.xml><?xml version="1.0" encoding="utf-8"?>
 <pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1" refreshedBy="hello" refreshedDate="45785.924756944398" createdVersion="5" refreshedVersion="5" minRefreshableVersion="3" recordCount="168">
   <cacheSource type="worksheet">
-    <worksheetSource ref="A1:G169" sheet="Sheet1"/>
+    <worksheetSource ref="A1:F169" sheet="Sheet1"/>
   </cacheSource>
   <cacheFields count="7">
     <cacheField name="时间戳" numFmtId="0">
@@ -2625,7 +2629,7 @@
 
 <file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
 <pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" name="PivotTable1" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="5" minRefreshableVersion="3" useAutoFormatting="1" createdVersion="5" indent="0" compact="0" outline="1" outlineData="1" compactData="0" multipleFieldFilters="0">
-  <location ref="K9:N25" firstHeaderRow="0" firstDataRow="1" firstDataCol="1"/>
+  <location ref="J9:M25" firstHeaderRow="0" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="7">
     <pivotField compact="0" showAll="0"/>
     <pivotField compact="0" showAll="0"/>
@@ -3270,16 +3274,16 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr filterMode="1"/>
-  <dimension ref="A1:N169"/>
+  <dimension ref="A1:M169"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5"/>
   <cols>
     <col min="1" max="1" width="17.375" style="1" customWidth="1"/>
     <col min="2" max="6" width="8.75" style="1"/>
-    <col min="11" max="11" width="11.625"/>
-    <col min="12" max="14" width="20.125"/>
+    <col min="10" max="10" width="11.625"/>
+    <col min="11" max="13" width="20.125"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14">
+    <row r="1" spans="1:13">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -3298,11 +3302,11 @@
       <c r="F1" s="7" t="s">
         <v>151</v>
       </c>
-      <c r="G1" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="2" spans="1:14" hidden="1">
+      <c r="G1" s="7" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="2" spans="1:13" hidden="1">
       <c r="A2" s="1" t="s">
         <v>6</v>
       </c>
@@ -3315,12 +3319,8 @@
       <c r="F2" s="1">
         <v>0.8</v>
       </c>
-      <c r="G2" t="str">
-        <f>RIGHT(A2,5)</f>
-        <v>00:00</v>
-      </c>
-    </row>
-    <row r="3" spans="1:14" hidden="1">
+    </row>
+    <row r="3" spans="1:13" hidden="1">
       <c r="A3" s="1" t="s">
         <v>7</v>
       </c>
@@ -3333,12 +3333,8 @@
       <c r="F3" s="1">
         <v>0.5</v>
       </c>
-      <c r="G3" t="str">
-        <f t="shared" ref="G3:G47" si="0">RIGHT(A3,5)</f>
-        <v>06:00</v>
-      </c>
-    </row>
-    <row r="4" spans="1:14">
+    </row>
+    <row r="4" spans="1:13">
       <c r="A4" s="1" t="s">
         <v>8</v>
       </c>
@@ -3349,11 +3345,11 @@
         <v>0.89</v>
       </c>
       <c r="G4" t="str">
-        <f t="shared" si="0"/>
-        <v>07:00</v>
-      </c>
-    </row>
-    <row r="5" spans="1:14" hidden="1">
+        <f>TEXT(A2,"HH:MM")</f>
+        <v>00:00</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13" hidden="1">
       <c r="A5" s="1" t="s">
         <v>8</v>
       </c>
@@ -3363,12 +3359,8 @@
       <c r="F5" s="1">
         <v>0.69</v>
       </c>
-      <c r="G5" t="str">
-        <f t="shared" si="0"/>
-        <v>07:00</v>
-      </c>
-    </row>
-    <row r="6" spans="1:14" hidden="1">
+    </row>
+    <row r="6" spans="1:13" hidden="1">
       <c r="A6" s="1" t="s">
         <v>9</v>
       </c>
@@ -3381,42 +3373,38 @@
       <c r="F6" s="1">
         <v>0.56999999999999995</v>
       </c>
-      <c r="G6" t="str">
+    </row>
+    <row r="7" spans="1:13">
+      <c r="A7" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D7" s="1">
+        <v>7.71</v>
+      </c>
+      <c r="F7" s="1">
+        <v>0.74</v>
+      </c>
+      <c r="G7" t="str">
+        <f t="shared" ref="G7:G8" si="0">TEXT(A5,"HH:MM")</f>
+        <v>07:00</v>
+      </c>
+    </row>
+    <row r="8" spans="1:13">
+      <c r="A8" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D8" s="1">
+        <v>6.46</v>
+      </c>
+      <c r="F8" s="1">
+        <v>0.7</v>
+      </c>
+      <c r="G8" t="str">
         <f t="shared" si="0"/>
         <v>07:30</v>
       </c>
     </row>
-    <row r="7" spans="1:14">
-      <c r="A7" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="D7" s="1">
-        <v>7.71</v>
-      </c>
-      <c r="F7" s="1">
-        <v>0.74</v>
-      </c>
-      <c r="G7" t="str">
-        <f t="shared" si="0"/>
-        <v>08:00</v>
-      </c>
-    </row>
-    <row r="8" spans="1:14">
-      <c r="A8" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="D8" s="1">
-        <v>6.46</v>
-      </c>
-      <c r="F8" s="1">
-        <v>0.7</v>
-      </c>
-      <c r="G8" t="str">
-        <f t="shared" si="0"/>
-        <v>09:00</v>
-      </c>
-    </row>
-    <row r="9" spans="1:14" hidden="1">
+    <row r="9" spans="1:13" hidden="1">
       <c r="A9" s="1" t="s">
         <v>12</v>
       </c>
@@ -3429,24 +3417,20 @@
       <c r="F9" s="1">
         <v>0.78</v>
       </c>
-      <c r="G9" t="str">
-        <f t="shared" si="0"/>
-        <v>10:00</v>
+      <c r="J9" t="s">
+        <v>5</v>
       </c>
       <c r="K9" t="s">
-        <v>5</v>
+        <v>13</v>
       </c>
       <c r="L9" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="M9" t="s">
-        <v>14</v>
-      </c>
-      <c r="N9" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="10" spans="1:14">
+    <row r="10" spans="1:13">
       <c r="A10" s="1" t="s">
         <v>16</v>
       </c>
@@ -3457,17 +3441,17 @@
         <v>0.47</v>
       </c>
       <c r="G10" t="str">
-        <f t="shared" si="0"/>
-        <v>12:00</v>
-      </c>
-      <c r="K10" t="s">
+        <f>TEXT(A8,"HH:MM")</f>
+        <v>09:00</v>
+      </c>
+      <c r="J10" t="s">
         <v>17</v>
       </c>
-      <c r="N10">
+      <c r="M10">
         <v>79.875</v>
       </c>
     </row>
-    <row r="11" spans="1:14" hidden="1">
+    <row r="11" spans="1:13" hidden="1">
       <c r="A11" s="1" t="s">
         <v>16</v>
       </c>
@@ -3480,18 +3464,14 @@
       <c r="F11" s="1">
         <v>0.99</v>
       </c>
-      <c r="G11" t="str">
-        <f t="shared" si="0"/>
-        <v>12:00</v>
-      </c>
-      <c r="K11" t="s">
+      <c r="J11" t="s">
         <v>18</v>
       </c>
-      <c r="N11">
+      <c r="M11">
         <v>81.375</v>
       </c>
     </row>
-    <row r="12" spans="1:14">
+    <row r="12" spans="1:13">
       <c r="A12" s="1" t="s">
         <v>19</v>
       </c>
@@ -3502,20 +3482,20 @@
         <v>0.51</v>
       </c>
       <c r="G12" t="str">
-        <f t="shared" si="0"/>
-        <v>13:00</v>
-      </c>
-      <c r="K12" t="s">
+        <f>TEXT(A10,"HH:MM")</f>
+        <v>12:00</v>
+      </c>
+      <c r="J12" t="s">
         <v>20</v>
       </c>
+      <c r="K12">
+        <v>4.4824999999999999</v>
+      </c>
       <c r="L12">
-        <v>4.4824999999999999</v>
-      </c>
-      <c r="M12">
         <v>0.17</v>
       </c>
     </row>
-    <row r="13" spans="1:14" hidden="1">
+    <row r="13" spans="1:13" hidden="1">
       <c r="A13" s="1" t="s">
         <v>19</v>
       </c>
@@ -3528,18 +3508,14 @@
       <c r="F13" s="1">
         <v>0.99</v>
       </c>
-      <c r="G13" t="str">
-        <f t="shared" si="0"/>
-        <v>13:00</v>
-      </c>
-      <c r="K13" t="s">
+      <c r="J13" t="s">
         <v>21</v>
       </c>
-      <c r="N13">
+      <c r="M13">
         <v>72.375</v>
       </c>
     </row>
-    <row r="14" spans="1:14">
+    <row r="14" spans="1:13">
       <c r="A14" s="1" t="s">
         <v>22</v>
       </c>
@@ -3550,17 +3526,17 @@
         <v>0.41</v>
       </c>
       <c r="G14" t="str">
-        <f t="shared" si="0"/>
-        <v>14:00</v>
-      </c>
-      <c r="K14" t="s">
+        <f>TEXT(A12,"HH:MM")</f>
+        <v>13:00</v>
+      </c>
+      <c r="J14" t="s">
         <v>23</v>
       </c>
-      <c r="L14">
+      <c r="K14">
         <v>6.8949999999999996</v>
       </c>
     </row>
-    <row r="15" spans="1:14" hidden="1">
+    <row r="15" spans="1:13" hidden="1">
       <c r="A15" s="1" t="s">
         <v>24</v>
       </c>
@@ -3573,18 +3549,14 @@
       <c r="F15" s="1">
         <v>0.95</v>
       </c>
-      <c r="G15" t="str">
-        <f t="shared" si="0"/>
-        <v>16:00</v>
-      </c>
-      <c r="K15" t="s">
+      <c r="J15" t="s">
         <v>25</v>
       </c>
-      <c r="L15">
+      <c r="K15">
         <v>5.9312500000000004</v>
       </c>
     </row>
-    <row r="16" spans="1:14">
+    <row r="16" spans="1:13">
       <c r="A16" s="1" t="s">
         <v>26</v>
       </c>
@@ -3595,17 +3567,17 @@
         <v>0.97</v>
       </c>
       <c r="G16" t="str">
-        <f t="shared" si="0"/>
-        <v>18:00</v>
-      </c>
-      <c r="K16" t="s">
+        <f>TEXT(A14,"HH:MM")</f>
+        <v>14:00</v>
+      </c>
+      <c r="J16" t="s">
         <v>27</v>
       </c>
-      <c r="N16">
+      <c r="M16">
         <v>72.5</v>
       </c>
     </row>
-    <row r="17" spans="1:14" hidden="1">
+    <row r="17" spans="1:13" hidden="1">
       <c r="A17" s="1" t="s">
         <v>26</v>
       </c>
@@ -3618,21 +3590,17 @@
       <c r="F17" s="1">
         <v>0.51</v>
       </c>
-      <c r="G17" t="str">
-        <f t="shared" si="0"/>
-        <v>18:00</v>
-      </c>
-      <c r="K17" t="s">
+      <c r="J17" t="s">
         <v>28</v>
       </c>
-      <c r="L17">
+      <c r="K17">
         <v>4.6387499999999999</v>
       </c>
-      <c r="N17">
+      <c r="M17">
         <v>70.25</v>
       </c>
     </row>
-    <row r="18" spans="1:14">
+    <row r="18" spans="1:13">
       <c r="A18" s="1" t="s">
         <v>29</v>
       </c>
@@ -3643,20 +3611,20 @@
         <v>0.54</v>
       </c>
       <c r="G18" t="str">
-        <f t="shared" si="0"/>
-        <v>19:00</v>
-      </c>
-      <c r="K18" t="s">
+        <f>TEXT(A16,"HH:MM")</f>
+        <v>18:00</v>
+      </c>
+      <c r="J18" t="s">
         <v>30</v>
       </c>
-      <c r="L18">
+      <c r="K18">
         <v>6.8125</v>
       </c>
-      <c r="N18">
+      <c r="M18">
         <v>72.5</v>
       </c>
     </row>
-    <row r="19" spans="1:14" hidden="1">
+    <row r="19" spans="1:13" hidden="1">
       <c r="A19" s="1" t="s">
         <v>29</v>
       </c>
@@ -3669,18 +3637,14 @@
       <c r="F19" s="1">
         <v>0.39</v>
       </c>
-      <c r="G19" t="str">
-        <f t="shared" si="0"/>
-        <v>19:00</v>
-      </c>
-      <c r="K19" t="s">
+      <c r="J19" t="s">
         <v>31</v>
       </c>
-      <c r="L19">
+      <c r="K19">
         <v>6.1987500000000004</v>
       </c>
     </row>
-    <row r="20" spans="1:14">
+    <row r="20" spans="1:13">
       <c r="A20" s="1" t="s">
         <v>32</v>
       </c>
@@ -3691,17 +3655,17 @@
         <v>0.66</v>
       </c>
       <c r="G20" t="str">
-        <f t="shared" si="0"/>
-        <v>20:00</v>
-      </c>
-      <c r="K20" t="s">
+        <f t="shared" ref="G20:G21" si="1">TEXT(A18,"HH:MM")</f>
+        <v>19:00</v>
+      </c>
+      <c r="J20" t="s">
         <v>33</v>
       </c>
-      <c r="N20">
+      <c r="M20">
         <v>73</v>
       </c>
     </row>
-    <row r="21" spans="1:14">
+    <row r="21" spans="1:13">
       <c r="A21" s="1" t="s">
         <v>34</v>
       </c>
@@ -3712,20 +3676,20 @@
         <v>0.66</v>
       </c>
       <c r="G21" t="str">
-        <f t="shared" si="0"/>
-        <v>22:00</v>
-      </c>
-      <c r="K21" t="s">
+        <f t="shared" si="1"/>
+        <v>19:00</v>
+      </c>
+      <c r="J21" t="s">
         <v>35</v>
       </c>
-      <c r="L21">
+      <c r="K21">
         <v>4.2712500000000002</v>
       </c>
-      <c r="N21">
+      <c r="M21">
         <v>77</v>
       </c>
     </row>
-    <row r="22" spans="1:14" hidden="1">
+    <row r="22" spans="1:13" hidden="1">
       <c r="A22" s="1" t="s">
         <v>34</v>
       </c>
@@ -3738,21 +3702,17 @@
       <c r="F22" s="1">
         <v>0.87</v>
       </c>
-      <c r="G22" t="str">
-        <f t="shared" si="0"/>
-        <v>22:00</v>
-      </c>
-      <c r="K22" t="s">
+      <c r="J22" t="s">
         <v>36</v>
       </c>
-      <c r="L22">
+      <c r="K22">
         <v>6.8087499999999999</v>
       </c>
-      <c r="N22">
+      <c r="M22">
         <v>74.375</v>
       </c>
     </row>
-    <row r="23" spans="1:14" hidden="1">
+    <row r="23" spans="1:13" hidden="1">
       <c r="A23" s="1" t="s">
         <v>37</v>
       </c>
@@ -3765,18 +3725,14 @@
       <c r="F23" s="1">
         <v>0.28000000000000003</v>
       </c>
-      <c r="G23" t="str">
-        <f t="shared" si="0"/>
-        <v>00:00</v>
-      </c>
-      <c r="K23" t="s">
+      <c r="J23" t="s">
         <v>38</v>
       </c>
-      <c r="L23">
+      <c r="K23">
         <v>5.8324999999999996</v>
       </c>
     </row>
-    <row r="24" spans="1:14" hidden="1">
+    <row r="24" spans="1:13" hidden="1">
       <c r="A24" s="1" t="s">
         <v>39</v>
       </c>
@@ -3789,21 +3745,17 @@
       <c r="F24" s="1">
         <v>0.37</v>
       </c>
-      <c r="G24" t="str">
-        <f t="shared" si="0"/>
-        <v>06:00</v>
-      </c>
-      <c r="K24" t="s">
+      <c r="J24" t="s">
         <v>40</v>
       </c>
-      <c r="L24">
+      <c r="K24">
         <v>4.5887500000000001</v>
       </c>
-      <c r="N24">
+      <c r="M24">
         <v>72</v>
       </c>
     </row>
-    <row r="25" spans="1:14">
+    <row r="25" spans="1:13">
       <c r="A25" s="1" t="s">
         <v>41</v>
       </c>
@@ -3814,23 +3766,23 @@
         <v>0.8</v>
       </c>
       <c r="G25" t="str">
-        <f t="shared" si="0"/>
-        <v>07:00</v>
-      </c>
-      <c r="K25" t="s">
+        <f>TEXT(A23,"HH:MM")</f>
+        <v>00:00</v>
+      </c>
+      <c r="J25" t="s">
         <v>42</v>
       </c>
+      <c r="K25">
+        <v>5.6459999999999999</v>
+      </c>
       <c r="L25">
-        <v>5.6459999999999999</v>
+        <v>0.17</v>
       </c>
       <c r="M25">
-        <v>0.17</v>
-      </c>
-      <c r="N25">
         <v>74.525000000000006</v>
       </c>
     </row>
-    <row r="26" spans="1:14" hidden="1">
+    <row r="26" spans="1:13" hidden="1">
       <c r="A26" s="1" t="s">
         <v>41</v>
       </c>
@@ -3840,12 +3792,8 @@
       <c r="F26" s="1">
         <v>0.65</v>
       </c>
-      <c r="G26" t="str">
-        <f t="shared" si="0"/>
-        <v>07:00</v>
-      </c>
-    </row>
-    <row r="27" spans="1:14" hidden="1">
+    </row>
+    <row r="27" spans="1:13" hidden="1">
       <c r="A27" s="1" t="s">
         <v>43</v>
       </c>
@@ -3858,12 +3806,8 @@
       <c r="F27" s="1">
         <v>0.23</v>
       </c>
-      <c r="G27" t="str">
-        <f t="shared" si="0"/>
-        <v>07:30</v>
-      </c>
-    </row>
-    <row r="28" spans="1:14">
+    </row>
+    <row r="28" spans="1:13">
       <c r="A28" s="1" t="s">
         <v>44</v>
       </c>
@@ -3874,11 +3818,11 @@
         <v>0.86</v>
       </c>
       <c r="G28" t="str">
-        <f t="shared" si="0"/>
-        <v>08:00</v>
-      </c>
-    </row>
-    <row r="29" spans="1:14">
+        <f t="shared" ref="G28:G29" si="2">TEXT(A26,"HH:MM")</f>
+        <v>07:00</v>
+      </c>
+    </row>
+    <row r="29" spans="1:13">
       <c r="A29" s="1" t="s">
         <v>45</v>
       </c>
@@ -3889,11 +3833,11 @@
         <v>0.51</v>
       </c>
       <c r="G29" t="str">
-        <f t="shared" si="0"/>
-        <v>09:00</v>
-      </c>
-    </row>
-    <row r="30" spans="1:14" hidden="1">
+        <f t="shared" si="2"/>
+        <v>07:30</v>
+      </c>
+    </row>
+    <row r="30" spans="1:13" hidden="1">
       <c r="A30" s="1" t="s">
         <v>46</v>
       </c>
@@ -3906,12 +3850,8 @@
       <c r="F30" s="1">
         <v>0.56000000000000005</v>
       </c>
-      <c r="G30" t="str">
-        <f t="shared" si="0"/>
-        <v>10:00</v>
-      </c>
-    </row>
-    <row r="31" spans="1:14">
+    </row>
+    <row r="31" spans="1:13">
       <c r="A31" s="1" t="s">
         <v>47</v>
       </c>
@@ -3922,11 +3862,11 @@
         <v>0.27</v>
       </c>
       <c r="G31" t="str">
-        <f t="shared" si="0"/>
-        <v>12:00</v>
-      </c>
-    </row>
-    <row r="32" spans="1:14" hidden="1">
+        <f>TEXT(A29,"HH:MM")</f>
+        <v>09:00</v>
+      </c>
+    </row>
+    <row r="32" spans="1:13" hidden="1">
       <c r="A32" s="1" t="s">
         <v>47</v>
       </c>
@@ -3938,10 +3878,6 @@
       </c>
       <c r="F32" s="1">
         <v>0.78</v>
-      </c>
-      <c r="G32" t="str">
-        <f t="shared" si="0"/>
-        <v>12:00</v>
       </c>
     </row>
     <row r="33" spans="1:7">
@@ -3955,8 +3891,8 @@
         <v>0.27</v>
       </c>
       <c r="G33" t="str">
-        <f t="shared" si="0"/>
-        <v>13:00</v>
+        <f>TEXT(A31,"HH:MM")</f>
+        <v>12:00</v>
       </c>
     </row>
     <row r="34" spans="1:7" hidden="1">
@@ -3972,10 +3908,6 @@
       <c r="F34" s="1">
         <v>0.8</v>
       </c>
-      <c r="G34" t="str">
-        <f t="shared" si="0"/>
-        <v>13:00</v>
-      </c>
     </row>
     <row r="35" spans="1:7">
       <c r="A35" s="1" t="s">
@@ -3988,8 +3920,8 @@
         <v>0.37</v>
       </c>
       <c r="G35" t="str">
-        <f t="shared" si="0"/>
-        <v>14:00</v>
+        <f>TEXT(A33,"HH:MM")</f>
+        <v>13:00</v>
       </c>
     </row>
     <row r="36" spans="1:7" hidden="1">
@@ -4005,10 +3937,6 @@
       <c r="F36" s="1">
         <v>0.33</v>
       </c>
-      <c r="G36" t="str">
-        <f t="shared" si="0"/>
-        <v>16:00</v>
-      </c>
     </row>
     <row r="37" spans="1:7">
       <c r="A37" s="1" t="s">
@@ -4021,8 +3949,8 @@
         <v>0.64</v>
       </c>
       <c r="G37" t="str">
-        <f t="shared" si="0"/>
-        <v>18:00</v>
+        <f>TEXT(A35,"HH:MM")</f>
+        <v>14:00</v>
       </c>
     </row>
     <row r="38" spans="1:7" hidden="1">
@@ -4038,10 +3966,6 @@
       <c r="F38" s="1">
         <v>0.85</v>
       </c>
-      <c r="G38" t="str">
-        <f t="shared" si="0"/>
-        <v>18:00</v>
-      </c>
     </row>
     <row r="39" spans="1:7">
       <c r="A39" s="1" t="s">
@@ -4054,8 +3978,8 @@
         <v>0.28000000000000003</v>
       </c>
       <c r="G39" t="str">
-        <f t="shared" si="0"/>
-        <v>19:00</v>
+        <f>TEXT(A37,"HH:MM")</f>
+        <v>18:00</v>
       </c>
     </row>
     <row r="40" spans="1:7" hidden="1">
@@ -4071,10 +3995,6 @@
       <c r="F40" s="1">
         <v>0.94</v>
       </c>
-      <c r="G40" t="str">
-        <f t="shared" si="0"/>
-        <v>19:00</v>
-      </c>
     </row>
     <row r="41" spans="1:7">
       <c r="A41" s="1" t="s">
@@ -4087,8 +4007,8 @@
         <v>0.32</v>
       </c>
       <c r="G41" t="str">
-        <f t="shared" si="0"/>
-        <v>20:00</v>
+        <f t="shared" ref="G41:G42" si="3">TEXT(A39,"HH:MM")</f>
+        <v>19:00</v>
       </c>
     </row>
     <row r="42" spans="1:7">
@@ -4102,8 +4022,8 @@
         <v>0.67</v>
       </c>
       <c r="G42" t="str">
-        <f t="shared" si="0"/>
-        <v>22:00</v>
+        <f t="shared" si="3"/>
+        <v>19:00</v>
       </c>
     </row>
     <row r="43" spans="1:7" hidden="1">
@@ -4119,10 +4039,6 @@
       <c r="F43" s="1">
         <v>0.88</v>
       </c>
-      <c r="G43" t="str">
-        <f t="shared" si="0"/>
-        <v>22:00</v>
-      </c>
     </row>
     <row r="44" spans="1:7" hidden="1">
       <c r="A44" s="1" t="s">
@@ -4137,10 +4053,6 @@
       <c r="F44" s="1">
         <v>0.41</v>
       </c>
-      <c r="G44" t="str">
-        <f t="shared" si="0"/>
-        <v>00:00</v>
-      </c>
     </row>
     <row r="45" spans="1:7" hidden="1">
       <c r="A45" s="1" t="s">
@@ -4155,10 +4067,6 @@
       <c r="F45" s="1">
         <v>0.65</v>
       </c>
-      <c r="G45" t="str">
-        <f t="shared" si="0"/>
-        <v>06:00</v>
-      </c>
     </row>
     <row r="46" spans="1:7">
       <c r="A46" s="1" t="s">
@@ -4171,8 +4079,8 @@
         <v>0.59</v>
       </c>
       <c r="G46" t="str">
-        <f t="shared" si="0"/>
-        <v>07:00</v>
+        <f>TEXT(A44,"HH:MM")</f>
+        <v>00:00</v>
       </c>
     </row>
     <row r="47" spans="1:7" hidden="1">
@@ -4185,10 +4093,6 @@
       <c r="F47" s="1">
         <v>0.68</v>
       </c>
-      <c r="G47" t="str">
-        <f t="shared" si="0"/>
-        <v>07:00</v>
-      </c>
     </row>
     <row r="48" spans="1:7" hidden="1">
       <c r="A48" s="1" t="s">
@@ -4203,10 +4107,6 @@
       <c r="F48" s="1">
         <v>0.6</v>
       </c>
-      <c r="G48" t="str">
-        <f t="shared" ref="G48:G79" si="1">RIGHT(A48,5)</f>
-        <v>07:30</v>
-      </c>
     </row>
     <row r="49" spans="1:7">
       <c r="A49" s="1" t="s">
@@ -4219,8 +4119,8 @@
         <v>0.76</v>
       </c>
       <c r="G49" t="str">
-        <f t="shared" si="1"/>
-        <v>08:00</v>
+        <f t="shared" ref="G49:G50" si="4">TEXT(A47,"HH:MM")</f>
+        <v>07:00</v>
       </c>
     </row>
     <row r="50" spans="1:7">
@@ -4234,8 +4134,8 @@
         <v>0.46</v>
       </c>
       <c r="G50" t="str">
-        <f t="shared" si="1"/>
-        <v>09:00</v>
+        <f t="shared" si="4"/>
+        <v>07:30</v>
       </c>
     </row>
     <row r="51" spans="1:7" hidden="1">
@@ -4251,10 +4151,6 @@
       <c r="F51" s="1">
         <v>0.61</v>
       </c>
-      <c r="G51" t="str">
-        <f t="shared" si="1"/>
-        <v>10:00</v>
-      </c>
     </row>
     <row r="52" spans="1:7">
       <c r="A52" s="1" t="s">
@@ -4267,8 +4163,8 @@
         <v>0.52</v>
       </c>
       <c r="G52" t="str">
-        <f t="shared" si="1"/>
-        <v>12:00</v>
+        <f>TEXT(A50,"HH:MM")</f>
+        <v>09:00</v>
       </c>
     </row>
     <row r="53" spans="1:7" hidden="1">
@@ -4284,10 +4180,6 @@
       <c r="F53" s="1">
         <v>0.53</v>
       </c>
-      <c r="G53" t="str">
-        <f t="shared" si="1"/>
-        <v>12:00</v>
-      </c>
     </row>
     <row r="54" spans="1:7">
       <c r="A54" s="1" t="s">
@@ -4300,8 +4192,8 @@
         <v>0.79</v>
       </c>
       <c r="G54" t="str">
-        <f t="shared" si="1"/>
-        <v>13:00</v>
+        <f>TEXT(A52,"HH:MM")</f>
+        <v>12:00</v>
       </c>
     </row>
     <row r="55" spans="1:7" hidden="1">
@@ -4317,10 +4209,6 @@
       <c r="F55" s="1">
         <v>0.44</v>
       </c>
-      <c r="G55" t="str">
-        <f t="shared" si="1"/>
-        <v>13:00</v>
-      </c>
     </row>
     <row r="56" spans="1:7">
       <c r="A56" s="1" t="s">
@@ -4333,8 +4221,8 @@
         <v>0.8</v>
       </c>
       <c r="G56" t="str">
-        <f t="shared" si="1"/>
-        <v>14:00</v>
+        <f>TEXT(A54,"HH:MM")</f>
+        <v>13:00</v>
       </c>
     </row>
     <row r="57" spans="1:7" hidden="1">
@@ -4350,10 +4238,6 @@
       <c r="F57" s="1">
         <v>0.45</v>
       </c>
-      <c r="G57" t="str">
-        <f t="shared" si="1"/>
-        <v>16:00</v>
-      </c>
     </row>
     <row r="58" spans="1:7">
       <c r="A58" s="1" t="s">
@@ -4366,8 +4250,8 @@
         <v>0.62</v>
       </c>
       <c r="G58" t="str">
-        <f t="shared" si="1"/>
-        <v>18:00</v>
+        <f>TEXT(A56,"HH:MM")</f>
+        <v>14:00</v>
       </c>
     </row>
     <row r="59" spans="1:7" hidden="1">
@@ -4383,10 +4267,6 @@
       <c r="F59" s="1">
         <v>0.61</v>
       </c>
-      <c r="G59" t="str">
-        <f t="shared" si="1"/>
-        <v>18:00</v>
-      </c>
     </row>
     <row r="60" spans="1:7">
       <c r="A60" s="1" t="s">
@@ -4399,8 +4279,8 @@
         <v>0.94</v>
       </c>
       <c r="G60" t="str">
-        <f t="shared" si="1"/>
-        <v>19:00</v>
+        <f>TEXT(A58,"HH:MM")</f>
+        <v>18:00</v>
       </c>
     </row>
     <row r="61" spans="1:7" hidden="1">
@@ -4416,10 +4296,6 @@
       <c r="F61" s="1">
         <v>0.65</v>
       </c>
-      <c r="G61" t="str">
-        <f t="shared" si="1"/>
-        <v>19:00</v>
-      </c>
     </row>
     <row r="62" spans="1:7">
       <c r="A62" s="1" t="s">
@@ -4432,8 +4308,8 @@
         <v>0.76</v>
       </c>
       <c r="G62" t="str">
-        <f t="shared" si="1"/>
-        <v>20:00</v>
+        <f t="shared" ref="G62:G63" si="5">TEXT(A60,"HH:MM")</f>
+        <v>19:00</v>
       </c>
     </row>
     <row r="63" spans="1:7">
@@ -4447,8 +4323,8 @@
         <v>0.51</v>
       </c>
       <c r="G63" t="str">
-        <f t="shared" si="1"/>
-        <v>22:00</v>
+        <f t="shared" si="5"/>
+        <v>19:00</v>
       </c>
     </row>
     <row r="64" spans="1:7" hidden="1">
@@ -4464,10 +4340,6 @@
       <c r="F64" s="1">
         <v>0.4</v>
       </c>
-      <c r="G64" t="str">
-        <f t="shared" si="1"/>
-        <v>22:00</v>
-      </c>
     </row>
     <row r="65" spans="1:7" hidden="1">
       <c r="A65" s="1" t="s">
@@ -4482,10 +4354,6 @@
       <c r="F65" s="1">
         <v>0.62</v>
       </c>
-      <c r="G65" t="str">
-        <f t="shared" si="1"/>
-        <v>00:00</v>
-      </c>
     </row>
     <row r="66" spans="1:7" hidden="1">
       <c r="A66" s="1" t="s">
@@ -4500,10 +4368,6 @@
       <c r="F66" s="1">
         <v>0.53</v>
       </c>
-      <c r="G66" t="str">
-        <f t="shared" si="1"/>
-        <v>06:00</v>
-      </c>
     </row>
     <row r="67" spans="1:7">
       <c r="A67" s="1" t="s">
@@ -4516,8 +4380,8 @@
         <v>0.42</v>
       </c>
       <c r="G67" t="str">
-        <f t="shared" si="1"/>
-        <v>07:00</v>
+        <f>TEXT(A65,"HH:MM")</f>
+        <v>00:00</v>
       </c>
     </row>
     <row r="68" spans="1:7" hidden="1">
@@ -4530,10 +4394,6 @@
       <c r="F68" s="1">
         <v>0.64</v>
       </c>
-      <c r="G68" t="str">
-        <f t="shared" si="1"/>
-        <v>07:00</v>
-      </c>
     </row>
     <row r="69" spans="1:7" hidden="1">
       <c r="A69" s="1" t="s">
@@ -4548,10 +4408,6 @@
       <c r="F69" s="1">
         <v>0.62</v>
       </c>
-      <c r="G69" t="str">
-        <f t="shared" si="1"/>
-        <v>07:30</v>
-      </c>
     </row>
     <row r="70" spans="1:7">
       <c r="A70" s="1" t="s">
@@ -4564,8 +4420,8 @@
         <v>0.48</v>
       </c>
       <c r="G70" t="str">
-        <f t="shared" si="1"/>
-        <v>08:00</v>
+        <f t="shared" ref="G70:G71" si="6">TEXT(A68,"HH:MM")</f>
+        <v>07:00</v>
       </c>
     </row>
     <row r="71" spans="1:7">
@@ -4579,8 +4435,8 @@
         <v>0.98</v>
       </c>
       <c r="G71" t="str">
-        <f t="shared" si="1"/>
-        <v>09:00</v>
+        <f t="shared" si="6"/>
+        <v>07:30</v>
       </c>
     </row>
     <row r="72" spans="1:7" hidden="1">
@@ -4596,10 +4452,6 @@
       <c r="F72" s="1">
         <v>0.64</v>
       </c>
-      <c r="G72" t="str">
-        <f t="shared" si="1"/>
-        <v>10:00</v>
-      </c>
     </row>
     <row r="73" spans="1:7">
       <c r="A73" s="1" t="s">
@@ -4612,8 +4464,8 @@
         <v>0.63</v>
       </c>
       <c r="G73" t="str">
-        <f t="shared" si="1"/>
-        <v>12:00</v>
+        <f>TEXT(A71,"HH:MM")</f>
+        <v>09:00</v>
       </c>
     </row>
     <row r="74" spans="1:7" hidden="1">
@@ -4629,10 +4481,6 @@
       <c r="F74" s="1">
         <v>0.49</v>
       </c>
-      <c r="G74" t="str">
-        <f t="shared" si="1"/>
-        <v>12:00</v>
-      </c>
     </row>
     <row r="75" spans="1:7">
       <c r="A75" s="1" t="s">
@@ -4645,8 +4493,8 @@
         <v>0.69</v>
       </c>
       <c r="G75" t="str">
-        <f t="shared" si="1"/>
-        <v>13:00</v>
+        <f>TEXT(A73,"HH:MM")</f>
+        <v>12:00</v>
       </c>
     </row>
     <row r="76" spans="1:7" hidden="1">
@@ -4662,10 +4510,6 @@
       <c r="F76" s="1">
         <v>0.71</v>
       </c>
-      <c r="G76" t="str">
-        <f t="shared" si="1"/>
-        <v>13:00</v>
-      </c>
     </row>
     <row r="77" spans="1:7">
       <c r="A77" s="1" t="s">
@@ -4678,8 +4522,8 @@
         <v>0.95</v>
       </c>
       <c r="G77" t="str">
-        <f t="shared" si="1"/>
-        <v>14:00</v>
+        <f>TEXT(A75,"HH:MM")</f>
+        <v>13:00</v>
       </c>
     </row>
     <row r="78" spans="1:7" hidden="1">
@@ -4695,10 +4539,6 @@
       <c r="F78" s="1">
         <v>0.89</v>
       </c>
-      <c r="G78" t="str">
-        <f t="shared" si="1"/>
-        <v>16:00</v>
-      </c>
     </row>
     <row r="79" spans="1:7">
       <c r="A79" s="1" t="s">
@@ -4711,8 +4551,8 @@
         <v>0.22</v>
       </c>
       <c r="G79" t="str">
-        <f t="shared" si="1"/>
-        <v>18:00</v>
+        <f>TEXT(A77,"HH:MM")</f>
+        <v>14:00</v>
       </c>
     </row>
     <row r="80" spans="1:7" hidden="1">
@@ -4728,10 +4568,6 @@
       <c r="F80" s="1">
         <v>0.77</v>
       </c>
-      <c r="G80" t="str">
-        <f t="shared" ref="G80:G111" si="2">RIGHT(A80,5)</f>
-        <v>18:00</v>
-      </c>
     </row>
     <row r="81" spans="1:7">
       <c r="A81" s="1" t="s">
@@ -4744,8 +4580,8 @@
         <v>0.8</v>
       </c>
       <c r="G81" t="str">
-        <f t="shared" si="2"/>
-        <v>19:00</v>
+        <f>TEXT(A79,"HH:MM")</f>
+        <v>18:00</v>
       </c>
     </row>
     <row r="82" spans="1:7" hidden="1">
@@ -4761,10 +4597,6 @@
       <c r="F82" s="1">
         <v>0.95</v>
       </c>
-      <c r="G82" t="str">
-        <f t="shared" si="2"/>
-        <v>19:00</v>
-      </c>
     </row>
     <row r="83" spans="1:7">
       <c r="A83" s="1" t="s">
@@ -4777,8 +4609,8 @@
         <v>0.23</v>
       </c>
       <c r="G83" t="str">
-        <f t="shared" si="2"/>
-        <v>20:00</v>
+        <f t="shared" ref="G83:G84" si="7">TEXT(A81,"HH:MM")</f>
+        <v>19:00</v>
       </c>
     </row>
     <row r="84" spans="1:7">
@@ -4792,8 +4624,8 @@
         <v>0.63</v>
       </c>
       <c r="G84" t="str">
-        <f t="shared" si="2"/>
-        <v>22:00</v>
+        <f t="shared" si="7"/>
+        <v>19:00</v>
       </c>
     </row>
     <row r="85" spans="1:7" hidden="1">
@@ -4809,10 +4641,6 @@
       <c r="F85" s="1">
         <v>0.73</v>
       </c>
-      <c r="G85" t="str">
-        <f t="shared" si="2"/>
-        <v>22:00</v>
-      </c>
     </row>
     <row r="86" spans="1:7" hidden="1">
       <c r="A86" s="1" t="s">
@@ -4827,10 +4655,6 @@
       <c r="F86" s="1">
         <v>0.63</v>
       </c>
-      <c r="G86" t="str">
-        <f t="shared" si="2"/>
-        <v>00:00</v>
-      </c>
     </row>
     <row r="87" spans="1:7" hidden="1">
       <c r="A87" s="1" t="s">
@@ -4845,10 +4669,6 @@
       <c r="F87" s="1">
         <v>0.92</v>
       </c>
-      <c r="G87" t="str">
-        <f t="shared" si="2"/>
-        <v>06:00</v>
-      </c>
     </row>
     <row r="88" spans="1:7">
       <c r="A88" s="1" t="s">
@@ -4861,8 +4681,8 @@
         <v>0.78</v>
       </c>
       <c r="G88" t="str">
-        <f t="shared" si="2"/>
-        <v>07:00</v>
+        <f>TEXT(A86,"HH:MM")</f>
+        <v>00:00</v>
       </c>
     </row>
     <row r="89" spans="1:7" hidden="1">
@@ -4875,10 +4695,6 @@
       <c r="F89" s="1">
         <v>0.66</v>
       </c>
-      <c r="G89" t="str">
-        <f t="shared" si="2"/>
-        <v>07:00</v>
-      </c>
     </row>
     <row r="90" spans="1:7" hidden="1">
       <c r="A90" s="1" t="s">
@@ -4893,10 +4709,6 @@
       <c r="F90" s="1">
         <v>0.82</v>
       </c>
-      <c r="G90" t="str">
-        <f t="shared" si="2"/>
-        <v>07:30</v>
-      </c>
     </row>
     <row r="91" spans="1:7">
       <c r="A91" s="1" t="s">
@@ -4909,8 +4721,8 @@
         <v>0.39</v>
       </c>
       <c r="G91" t="str">
-        <f t="shared" si="2"/>
-        <v>08:00</v>
+        <f t="shared" ref="G91:G92" si="8">TEXT(A89,"HH:MM")</f>
+        <v>07:00</v>
       </c>
     </row>
     <row r="92" spans="1:7">
@@ -4924,8 +4736,8 @@
         <v>0.69</v>
       </c>
       <c r="G92" t="str">
-        <f t="shared" si="2"/>
-        <v>09:00</v>
+        <f t="shared" si="8"/>
+        <v>07:30</v>
       </c>
     </row>
     <row r="93" spans="1:7" hidden="1">
@@ -4941,10 +4753,6 @@
       <c r="F93" s="1">
         <v>0.27</v>
       </c>
-      <c r="G93" t="str">
-        <f t="shared" si="2"/>
-        <v>10:00</v>
-      </c>
     </row>
     <row r="94" spans="1:7">
       <c r="A94" s="1" t="s">
@@ -4957,8 +4765,8 @@
         <v>0.74</v>
       </c>
       <c r="G94" t="str">
-        <f t="shared" si="2"/>
-        <v>12:00</v>
+        <f>TEXT(A92,"HH:MM")</f>
+        <v>09:00</v>
       </c>
     </row>
     <row r="95" spans="1:7" hidden="1">
@@ -4974,10 +4782,6 @@
       <c r="F95" s="1">
         <v>0.92</v>
       </c>
-      <c r="G95" t="str">
-        <f t="shared" si="2"/>
-        <v>12:00</v>
-      </c>
     </row>
     <row r="96" spans="1:7">
       <c r="A96" s="1" t="s">
@@ -4990,8 +4794,8 @@
         <v>0.82</v>
       </c>
       <c r="G96" t="str">
-        <f t="shared" si="2"/>
-        <v>13:00</v>
+        <f>TEXT(A94,"HH:MM")</f>
+        <v>12:00</v>
       </c>
     </row>
     <row r="97" spans="1:7" hidden="1">
@@ -5007,10 +4811,6 @@
       <c r="F97" s="1">
         <v>0.21</v>
       </c>
-      <c r="G97" t="str">
-        <f t="shared" si="2"/>
-        <v>13:00</v>
-      </c>
     </row>
     <row r="98" spans="1:7">
       <c r="A98" s="1" t="s">
@@ -5023,8 +4823,8 @@
         <v>0.27</v>
       </c>
       <c r="G98" t="str">
-        <f t="shared" si="2"/>
-        <v>14:00</v>
+        <f>TEXT(A96,"HH:MM")</f>
+        <v>13:00</v>
       </c>
     </row>
     <row r="99" spans="1:7" hidden="1">
@@ -5040,10 +4840,6 @@
       <c r="F99" s="1">
         <v>0.2</v>
       </c>
-      <c r="G99" t="str">
-        <f t="shared" si="2"/>
-        <v>16:00</v>
-      </c>
     </row>
     <row r="100" spans="1:7">
       <c r="A100" s="1" t="s">
@@ -5056,8 +4852,8 @@
         <v>0.76</v>
       </c>
       <c r="G100" t="str">
-        <f t="shared" si="2"/>
-        <v>18:00</v>
+        <f>TEXT(A98,"HH:MM")</f>
+        <v>14:00</v>
       </c>
     </row>
     <row r="101" spans="1:7" hidden="1">
@@ -5073,10 +4869,6 @@
       <c r="F101" s="1">
         <v>0.64</v>
       </c>
-      <c r="G101" t="str">
-        <f t="shared" si="2"/>
-        <v>18:00</v>
-      </c>
     </row>
     <row r="102" spans="1:7">
       <c r="A102" s="1" t="s">
@@ -5089,8 +4881,8 @@
         <v>0.71</v>
       </c>
       <c r="G102" t="str">
-        <f t="shared" si="2"/>
-        <v>19:00</v>
+        <f>TEXT(A100,"HH:MM")</f>
+        <v>18:00</v>
       </c>
     </row>
     <row r="103" spans="1:7" hidden="1">
@@ -5106,10 +4898,6 @@
       <c r="F103" s="1">
         <v>0.38</v>
       </c>
-      <c r="G103" t="str">
-        <f t="shared" si="2"/>
-        <v>19:00</v>
-      </c>
     </row>
     <row r="104" spans="1:7">
       <c r="A104" s="1" t="s">
@@ -5122,8 +4910,8 @@
         <v>0.93</v>
       </c>
       <c r="G104" t="str">
-        <f t="shared" si="2"/>
-        <v>20:00</v>
+        <f t="shared" ref="G104:G105" si="9">TEXT(A102,"HH:MM")</f>
+        <v>19:00</v>
       </c>
     </row>
     <row r="105" spans="1:7">
@@ -5137,8 +4925,8 @@
         <v>0.76</v>
       </c>
       <c r="G105" t="str">
-        <f t="shared" si="2"/>
-        <v>22:00</v>
+        <f t="shared" si="9"/>
+        <v>19:00</v>
       </c>
     </row>
     <row r="106" spans="1:7" hidden="1">
@@ -5154,10 +4942,6 @@
       <c r="F106" s="1">
         <v>0.49</v>
       </c>
-      <c r="G106" t="str">
-        <f t="shared" si="2"/>
-        <v>22:00</v>
-      </c>
     </row>
     <row r="107" spans="1:7" hidden="1">
       <c r="A107" s="1" t="s">
@@ -5172,10 +4956,6 @@
       <c r="F107" s="1">
         <v>0.88</v>
       </c>
-      <c r="G107" t="str">
-        <f t="shared" si="2"/>
-        <v>00:00</v>
-      </c>
     </row>
     <row r="108" spans="1:7" hidden="1">
       <c r="A108" s="1" t="s">
@@ -5190,10 +4970,6 @@
       <c r="F108" s="1">
         <v>0.92</v>
       </c>
-      <c r="G108" t="str">
-        <f t="shared" si="2"/>
-        <v>06:00</v>
-      </c>
     </row>
     <row r="109" spans="1:7">
       <c r="A109" s="1" t="s">
@@ -5206,8 +4982,8 @@
         <v>0.56999999999999995</v>
       </c>
       <c r="G109" t="str">
-        <f t="shared" si="2"/>
-        <v>07:00</v>
+        <f>TEXT(A107,"HH:MM")</f>
+        <v>00:00</v>
       </c>
     </row>
     <row r="110" spans="1:7" hidden="1">
@@ -5220,10 +4996,6 @@
       <c r="F110" s="1">
         <v>0.63</v>
       </c>
-      <c r="G110" t="str">
-        <f t="shared" si="2"/>
-        <v>07:00</v>
-      </c>
     </row>
     <row r="111" spans="1:7" hidden="1">
       <c r="A111" s="1" t="s">
@@ -5238,10 +5010,6 @@
       <c r="F111" s="1">
         <v>0.36</v>
       </c>
-      <c r="G111" t="str">
-        <f t="shared" si="2"/>
-        <v>07:30</v>
-      </c>
     </row>
     <row r="112" spans="1:7">
       <c r="A112" s="1" t="s">
@@ -5254,8 +5022,8 @@
         <v>0.59</v>
       </c>
       <c r="G112" t="str">
-        <f t="shared" ref="G112:G143" si="3">RIGHT(A112,5)</f>
-        <v>08:00</v>
+        <f t="shared" ref="G112:G113" si="10">TEXT(A110,"HH:MM")</f>
+        <v>07:00</v>
       </c>
     </row>
     <row r="113" spans="1:7">
@@ -5269,8 +5037,8 @@
         <v>0.76</v>
       </c>
       <c r="G113" t="str">
-        <f t="shared" si="3"/>
-        <v>09:00</v>
+        <f t="shared" si="10"/>
+        <v>07:30</v>
       </c>
     </row>
     <row r="114" spans="1:7" hidden="1">
@@ -5286,10 +5054,6 @@
       <c r="F114" s="1">
         <v>0.23</v>
       </c>
-      <c r="G114" t="str">
-        <f t="shared" si="3"/>
-        <v>10:00</v>
-      </c>
     </row>
     <row r="115" spans="1:7">
       <c r="A115" s="1" t="s">
@@ -5302,8 +5066,8 @@
         <v>0.76</v>
       </c>
       <c r="G115" t="str">
-        <f t="shared" si="3"/>
-        <v>12:00</v>
+        <f>TEXT(A113,"HH:MM")</f>
+        <v>09:00</v>
       </c>
     </row>
     <row r="116" spans="1:7" hidden="1">
@@ -5319,10 +5083,6 @@
       <c r="F116" s="1">
         <v>0.57999999999999996</v>
       </c>
-      <c r="G116" t="str">
-        <f t="shared" si="3"/>
-        <v>12:00</v>
-      </c>
     </row>
     <row r="117" spans="1:7">
       <c r="A117" s="1" t="s">
@@ -5335,8 +5095,8 @@
         <v>0.48</v>
       </c>
       <c r="G117" t="str">
-        <f t="shared" si="3"/>
-        <v>13:00</v>
+        <f>TEXT(A115,"HH:MM")</f>
+        <v>12:00</v>
       </c>
     </row>
     <row r="118" spans="1:7" hidden="1">
@@ -5352,10 +5112,6 @@
       <c r="F118" s="1">
         <v>0.8</v>
       </c>
-      <c r="G118" t="str">
-        <f t="shared" si="3"/>
-        <v>13:00</v>
-      </c>
     </row>
     <row r="119" spans="1:7">
       <c r="A119" s="1" t="s">
@@ -5368,8 +5124,8 @@
         <v>0.63</v>
       </c>
       <c r="G119" t="str">
-        <f t="shared" si="3"/>
-        <v>14:00</v>
+        <f>TEXT(A117,"HH:MM")</f>
+        <v>13:00</v>
       </c>
     </row>
     <row r="120" spans="1:7" hidden="1">
@@ -5385,10 +5141,6 @@
       <c r="F120" s="1">
         <v>0.98</v>
       </c>
-      <c r="G120" t="str">
-        <f t="shared" si="3"/>
-        <v>16:00</v>
-      </c>
     </row>
     <row r="121" spans="1:7">
       <c r="A121" s="1" t="s">
@@ -5401,8 +5153,8 @@
         <v>0.3</v>
       </c>
       <c r="G121" t="str">
-        <f t="shared" si="3"/>
-        <v>18:00</v>
+        <f>TEXT(A119,"HH:MM")</f>
+        <v>14:00</v>
       </c>
     </row>
     <row r="122" spans="1:7" hidden="1">
@@ -5418,10 +5170,6 @@
       <c r="F122" s="1">
         <v>0.35</v>
       </c>
-      <c r="G122" t="str">
-        <f t="shared" si="3"/>
-        <v>18:00</v>
-      </c>
     </row>
     <row r="123" spans="1:7">
       <c r="A123" s="1" t="s">
@@ -5434,8 +5182,8 @@
         <v>0.27</v>
       </c>
       <c r="G123" t="str">
-        <f t="shared" si="3"/>
-        <v>19:00</v>
+        <f>TEXT(A121,"HH:MM")</f>
+        <v>18:00</v>
       </c>
     </row>
     <row r="124" spans="1:7" hidden="1">
@@ -5451,10 +5199,6 @@
       <c r="F124" s="1">
         <v>0.94</v>
       </c>
-      <c r="G124" t="str">
-        <f t="shared" si="3"/>
-        <v>19:00</v>
-      </c>
     </row>
     <row r="125" spans="1:7">
       <c r="A125" s="1" t="s">
@@ -5467,8 +5211,8 @@
         <v>0.8</v>
       </c>
       <c r="G125" t="str">
-        <f t="shared" si="3"/>
-        <v>20:00</v>
+        <f t="shared" ref="G125:G126" si="11">TEXT(A123,"HH:MM")</f>
+        <v>19:00</v>
       </c>
     </row>
     <row r="126" spans="1:7">
@@ -5482,8 +5226,8 @@
         <v>0.39</v>
       </c>
       <c r="G126" t="str">
-        <f t="shared" si="3"/>
-        <v>22:00</v>
+        <f t="shared" si="11"/>
+        <v>19:00</v>
       </c>
     </row>
     <row r="127" spans="1:7" hidden="1">
@@ -5499,10 +5243,6 @@
       <c r="F127" s="1">
         <v>0.37</v>
       </c>
-      <c r="G127" t="str">
-        <f t="shared" si="3"/>
-        <v>22:00</v>
-      </c>
     </row>
     <row r="128" spans="1:7" hidden="1">
       <c r="A128" s="1" t="s">
@@ -5517,10 +5257,6 @@
       <c r="F128" s="1">
         <v>0.63</v>
       </c>
-      <c r="G128" t="str">
-        <f t="shared" si="3"/>
-        <v>00:00</v>
-      </c>
     </row>
     <row r="129" spans="1:7" hidden="1">
       <c r="A129" s="1" t="s">
@@ -5535,10 +5271,6 @@
       <c r="F129" s="1">
         <v>0.69</v>
       </c>
-      <c r="G129" t="str">
-        <f t="shared" si="3"/>
-        <v>06:00</v>
-      </c>
     </row>
     <row r="130" spans="1:7">
       <c r="A130" s="1" t="s">
@@ -5551,8 +5283,8 @@
         <v>0.78</v>
       </c>
       <c r="G130" t="str">
-        <f t="shared" si="3"/>
-        <v>07:00</v>
+        <f>TEXT(A128,"HH:MM")</f>
+        <v>00:00</v>
       </c>
     </row>
     <row r="131" spans="1:7" hidden="1">
@@ -5565,10 +5297,6 @@
       <c r="F131" s="1">
         <v>0.68</v>
       </c>
-      <c r="G131" t="str">
-        <f t="shared" si="3"/>
-        <v>07:00</v>
-      </c>
     </row>
     <row r="132" spans="1:7" hidden="1">
       <c r="A132" s="1" t="s">
@@ -5583,10 +5311,6 @@
       <c r="F132" s="1">
         <v>0.2</v>
       </c>
-      <c r="G132" t="str">
-        <f t="shared" si="3"/>
-        <v>07:30</v>
-      </c>
     </row>
     <row r="133" spans="1:7">
       <c r="A133" s="1" t="s">
@@ -5599,8 +5323,8 @@
         <v>0.32</v>
       </c>
       <c r="G133" t="str">
-        <f t="shared" si="3"/>
-        <v>08:00</v>
+        <f t="shared" ref="G133:G134" si="12">TEXT(A131,"HH:MM")</f>
+        <v>07:00</v>
       </c>
     </row>
     <row r="134" spans="1:7">
@@ -5614,8 +5338,8 @@
         <v>0.63</v>
       </c>
       <c r="G134" t="str">
-        <f t="shared" si="3"/>
-        <v>09:00</v>
+        <f t="shared" si="12"/>
+        <v>07:30</v>
       </c>
     </row>
     <row r="135" spans="1:7" hidden="1">
@@ -5631,10 +5355,6 @@
       <c r="F135" s="1">
         <v>0.26</v>
       </c>
-      <c r="G135" t="str">
-        <f t="shared" si="3"/>
-        <v>10:00</v>
-      </c>
     </row>
     <row r="136" spans="1:7">
       <c r="A136" s="1" t="s">
@@ -5647,8 +5367,8 @@
         <v>0.65</v>
       </c>
       <c r="G136" t="str">
-        <f t="shared" si="3"/>
-        <v>12:00</v>
+        <f>TEXT(A134,"HH:MM")</f>
+        <v>09:00</v>
       </c>
     </row>
     <row r="137" spans="1:7" hidden="1">
@@ -5664,10 +5384,6 @@
       <c r="F137" s="1">
         <v>0.91</v>
       </c>
-      <c r="G137" t="str">
-        <f t="shared" si="3"/>
-        <v>12:00</v>
-      </c>
     </row>
     <row r="138" spans="1:7">
       <c r="A138" s="1" t="s">
@@ -5680,8 +5396,8 @@
         <v>0.57999999999999996</v>
       </c>
       <c r="G138" t="str">
-        <f t="shared" si="3"/>
-        <v>13:00</v>
+        <f>TEXT(A136,"HH:MM")</f>
+        <v>12:00</v>
       </c>
     </row>
     <row r="139" spans="1:7" hidden="1">
@@ -5697,10 +5413,6 @@
       <c r="F139" s="1">
         <v>0.99</v>
       </c>
-      <c r="G139" t="str">
-        <f t="shared" si="3"/>
-        <v>13:00</v>
-      </c>
     </row>
     <row r="140" spans="1:7">
       <c r="A140" s="1" t="s">
@@ -5713,8 +5425,8 @@
         <v>0.57999999999999996</v>
       </c>
       <c r="G140" t="str">
-        <f t="shared" si="3"/>
-        <v>14:00</v>
+        <f>TEXT(A138,"HH:MM")</f>
+        <v>13:00</v>
       </c>
     </row>
     <row r="141" spans="1:7" hidden="1">
@@ -5730,10 +5442,6 @@
       <c r="F141" s="1">
         <v>0.89</v>
       </c>
-      <c r="G141" t="str">
-        <f t="shared" si="3"/>
-        <v>16:00</v>
-      </c>
     </row>
     <row r="142" spans="1:7">
       <c r="A142" s="1" t="s">
@@ -5746,8 +5454,8 @@
         <v>0.65</v>
       </c>
       <c r="G142" t="str">
-        <f t="shared" si="3"/>
-        <v>18:00</v>
+        <f>TEXT(A140,"HH:MM")</f>
+        <v>14:00</v>
       </c>
     </row>
     <row r="143" spans="1:7" hidden="1">
@@ -5763,10 +5471,6 @@
       <c r="F143" s="1">
         <v>0.82</v>
       </c>
-      <c r="G143" t="str">
-        <f t="shared" si="3"/>
-        <v>18:00</v>
-      </c>
     </row>
     <row r="144" spans="1:7">
       <c r="A144" s="1" t="s">
@@ -5779,8 +5483,8 @@
         <v>0.47</v>
       </c>
       <c r="G144" t="str">
-        <f t="shared" ref="G144:G153" si="4">RIGHT(A144,5)</f>
-        <v>19:00</v>
+        <f>TEXT(A142,"HH:MM")</f>
+        <v>18:00</v>
       </c>
     </row>
     <row r="145" spans="1:7" hidden="1">
@@ -5796,10 +5500,6 @@
       <c r="F145" s="1">
         <v>0.7</v>
       </c>
-      <c r="G145" t="str">
-        <f t="shared" si="4"/>
-        <v>19:00</v>
-      </c>
     </row>
     <row r="146" spans="1:7">
       <c r="A146" s="1" t="s">
@@ -5812,8 +5512,8 @@
         <v>0.4</v>
       </c>
       <c r="G146" t="str">
-        <f t="shared" si="4"/>
-        <v>20:00</v>
+        <f t="shared" ref="G146:G147" si="13">TEXT(A144,"HH:MM")</f>
+        <v>19:00</v>
       </c>
     </row>
     <row r="147" spans="1:7">
@@ -5827,8 +5527,8 @@
         <v>0.49</v>
       </c>
       <c r="G147" t="str">
-        <f t="shared" si="4"/>
-        <v>22:00</v>
+        <f t="shared" si="13"/>
+        <v>19:00</v>
       </c>
     </row>
     <row r="148" spans="1:7" hidden="1">
@@ -5844,10 +5544,6 @@
       <c r="F148" s="1">
         <v>0.24</v>
       </c>
-      <c r="G148" t="str">
-        <f t="shared" si="4"/>
-        <v>22:00</v>
-      </c>
     </row>
     <row r="149" spans="1:7" hidden="1">
       <c r="A149" s="1" t="s">
@@ -5862,10 +5558,6 @@
       <c r="F149" s="1">
         <v>0.69</v>
       </c>
-      <c r="G149" t="str">
-        <f t="shared" si="4"/>
-        <v>00:00</v>
-      </c>
     </row>
     <row r="150" spans="1:7" hidden="1">
       <c r="A150" s="1" t="s">
@@ -5880,10 +5572,6 @@
       <c r="F150" s="1">
         <v>0.46</v>
       </c>
-      <c r="G150" t="str">
-        <f t="shared" si="4"/>
-        <v>06:00</v>
-      </c>
     </row>
     <row r="151" spans="1:7">
       <c r="A151" s="1" t="s">
@@ -5896,8 +5584,8 @@
         <v>0.88</v>
       </c>
       <c r="G151" t="str">
-        <f t="shared" si="4"/>
-        <v>07:00</v>
+        <f>TEXT(A149,"HH:MM")</f>
+        <v>00:00</v>
       </c>
     </row>
     <row r="152" spans="1:7" hidden="1">
@@ -5910,10 +5598,6 @@
       <c r="F152" s="1">
         <v>0.66</v>
       </c>
-      <c r="G152" t="str">
-        <f t="shared" si="4"/>
-        <v>07:00</v>
-      </c>
     </row>
     <row r="153" spans="1:7" hidden="1">
       <c r="A153" s="1" t="s">
@@ -5928,10 +5612,6 @@
       <c r="F153" s="1">
         <v>0.4</v>
       </c>
-      <c r="G153" t="str">
-        <f t="shared" si="4"/>
-        <v>07:30</v>
-      </c>
     </row>
     <row r="154" spans="1:7">
       <c r="A154" s="1" t="s">
@@ -5944,8 +5624,8 @@
         <v>0.84</v>
       </c>
       <c r="G154" t="str">
-        <f t="shared" ref="G154:G169" si="5">RIGHT(A154,5)</f>
-        <v>08:00</v>
+        <f t="shared" ref="G154:G155" si="14">TEXT(A152,"HH:MM")</f>
+        <v>07:00</v>
       </c>
     </row>
     <row r="155" spans="1:7">
@@ -5959,8 +5639,8 @@
         <v>0.24</v>
       </c>
       <c r="G155" t="str">
-        <f t="shared" si="5"/>
-        <v>09:00</v>
+        <f t="shared" si="14"/>
+        <v>07:30</v>
       </c>
     </row>
     <row r="156" spans="1:7" hidden="1">
@@ -5976,10 +5656,6 @@
       <c r="F156" s="1">
         <v>0.54</v>
       </c>
-      <c r="G156" t="str">
-        <f t="shared" si="5"/>
-        <v>10:00</v>
-      </c>
     </row>
     <row r="157" spans="1:7">
       <c r="A157" s="1" t="s">
@@ -5992,8 +5668,8 @@
         <v>0.52</v>
       </c>
       <c r="G157" t="str">
-        <f t="shared" si="5"/>
-        <v>12:00</v>
+        <f>TEXT(A155,"HH:MM")</f>
+        <v>09:00</v>
       </c>
     </row>
     <row r="158" spans="1:7" hidden="1">
@@ -6009,10 +5685,6 @@
       <c r="F158" s="1">
         <v>0.93</v>
       </c>
-      <c r="G158" t="str">
-        <f t="shared" si="5"/>
-        <v>12:00</v>
-      </c>
     </row>
     <row r="159" spans="1:7">
       <c r="A159" s="1" t="s">
@@ -6025,8 +5697,8 @@
         <v>0.85</v>
       </c>
       <c r="G159" t="str">
-        <f t="shared" si="5"/>
-        <v>13:00</v>
+        <f>TEXT(A157,"HH:MM")</f>
+        <v>12:00</v>
       </c>
     </row>
     <row r="160" spans="1:7" hidden="1">
@@ -6042,10 +5714,6 @@
       <c r="F160" s="1">
         <v>0.71</v>
       </c>
-      <c r="G160" t="str">
-        <f t="shared" si="5"/>
-        <v>13:00</v>
-      </c>
     </row>
     <row r="161" spans="1:7">
       <c r="A161" s="1" t="s">
@@ -6058,8 +5726,8 @@
         <v>0.65</v>
       </c>
       <c r="G161" t="str">
-        <f t="shared" si="5"/>
-        <v>14:00</v>
+        <f>TEXT(A159,"HH:MM")</f>
+        <v>13:00</v>
       </c>
     </row>
     <row r="162" spans="1:7" hidden="1">
@@ -6075,10 +5743,6 @@
       <c r="F162" s="1">
         <v>0.28999999999999998</v>
       </c>
-      <c r="G162" t="str">
-        <f t="shared" si="5"/>
-        <v>16:00</v>
-      </c>
     </row>
     <row r="163" spans="1:7">
       <c r="A163" s="1" t="s">
@@ -6091,8 +5755,8 @@
         <v>0.42</v>
       </c>
       <c r="G163" t="str">
-        <f t="shared" si="5"/>
-        <v>18:00</v>
+        <f>TEXT(A161,"HH:MM")</f>
+        <v>14:00</v>
       </c>
     </row>
     <row r="164" spans="1:7" hidden="1">
@@ -6108,10 +5772,6 @@
       <c r="F164" s="1">
         <v>0.34</v>
       </c>
-      <c r="G164" t="str">
-        <f t="shared" si="5"/>
-        <v>18:00</v>
-      </c>
     </row>
     <row r="165" spans="1:7">
       <c r="A165" s="1" t="s">
@@ -6124,8 +5784,8 @@
         <v>0.54</v>
       </c>
       <c r="G165" t="str">
-        <f t="shared" si="5"/>
-        <v>19:00</v>
+        <f>TEXT(A163,"HH:MM")</f>
+        <v>18:00</v>
       </c>
     </row>
     <row r="166" spans="1:7" hidden="1">
@@ -6141,10 +5801,6 @@
       <c r="F166" s="1">
         <v>0.69</v>
       </c>
-      <c r="G166" t="str">
-        <f t="shared" si="5"/>
-        <v>19:00</v>
-      </c>
     </row>
     <row r="167" spans="1:7">
       <c r="A167" s="1" t="s">
@@ -6157,8 +5813,8 @@
         <v>0.27</v>
       </c>
       <c r="G167" t="str">
-        <f t="shared" si="5"/>
-        <v>20:00</v>
+        <f t="shared" ref="G167:G168" si="15">TEXT(A165,"HH:MM")</f>
+        <v>19:00</v>
       </c>
     </row>
     <row r="168" spans="1:7">
@@ -6172,8 +5828,8 @@
         <v>0.46</v>
       </c>
       <c r="G168" t="str">
-        <f t="shared" si="5"/>
-        <v>22:00</v>
+        <f t="shared" si="15"/>
+        <v>19:00</v>
       </c>
     </row>
     <row r="169" spans="1:7" hidden="1">
@@ -6188,10 +5844,6 @@
       </c>
       <c r="F169" s="1">
         <v>0.6</v>
-      </c>
-      <c r="G169" t="str">
-        <f t="shared" si="5"/>
-        <v>22:00</v>
       </c>
     </row>
   </sheetData>

</xml_diff>